<commit_message>
Regenerate grounding and prediction outputs after line reviews
Reruns the notebook/ari-grounding pipeline (parse_doid_local -> ground_doid ->
ground_snomed -> make_match_reports -> predict_target_matches ->
resolve_target_labels -> build_disease_target_matrix) against the current
ontology and SSSOM, so the predictions, labels and reports 5-8 reflect the
ARI#92-#96, #105 and #107 reviews merged since PR #104. No script changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/4-reports/7_SNOMED_Matches_All.xlsx
+++ b/data/4-reports/7_SNOMED_Matches_All.xlsx
@@ -693,7 +693,7 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>83942000, 72986009</t>
+          <t>83942000</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -1177,11 +1177,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>763803004</t>
-        </is>
-      </c>
+      <c r="J14" s="3" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
@@ -1728,7 +1724,7 @@
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>13445001, 232308006</t>
+          <t>232308006</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
@@ -1834,7 +1830,7 @@
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>452281000124106, 716684004</t>
+          <t>452281000124106</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
@@ -1940,7 +1936,7 @@
       <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>235728001, 84027009, 84568007</t>
+          <t>84568007</t>
         </is>
       </c>
       <c r="K31" s="5" t="inlineStr">
@@ -1993,7 +1989,7 @@
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>413603009, 718716008</t>
+          <t>413603009</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
@@ -2046,7 +2042,7 @@
       <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>721711009, 408335007, 16098491000119109, 721713007, 721712002</t>
+          <t>408335007</t>
         </is>
       </c>
       <c r="K33" s="5" t="inlineStr">
@@ -2440,14 +2436,10 @@
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr"/>
-      <c r="J41" s="3" t="inlineStr">
-        <is>
-          <t>721198006</t>
-        </is>
-      </c>
-      <c r="K41" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="J41" s="3" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>n/a (no existing code)</t>
         </is>
       </c>
     </row>
@@ -2548,7 +2540,7 @@
       <c r="I43" s="2" t="inlineStr"/>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>722872000, 1197740007, 448542008</t>
+          <t>448542008</t>
         </is>
       </c>
       <c r="K43" s="5" t="inlineStr">
@@ -3207,14 +3199,10 @@
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr"/>
-      <c r="J56" s="3" t="inlineStr">
-        <is>
-          <t>231981005</t>
-        </is>
-      </c>
-      <c r="K56" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
+      <c r="J56" s="3" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>n/a (no existing code)</t>
         </is>
       </c>
     </row>
@@ -4110,7 +4098,11 @@
       </c>
       <c r="H75" s="2" t="inlineStr"/>
       <c r="I75" s="2" t="inlineStr"/>
-      <c r="J75" s="3" t="inlineStr"/>
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t>1197361002</t>
+        </is>
+      </c>
       <c r="K75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
@@ -4316,7 +4308,7 @@
       <c r="I79" s="2" t="inlineStr"/>
       <c r="J79" s="3" t="inlineStr">
         <is>
-          <t>396230008, 1212005</t>
+          <t>396230008</t>
         </is>
       </c>
       <c r="K79" s="5" t="inlineStr">
@@ -4478,7 +4470,11 @@
       </c>
       <c r="H83" s="2" t="inlineStr"/>
       <c r="I83" s="2" t="inlineStr"/>
-      <c r="J83" s="3" t="inlineStr"/>
+      <c r="J83" s="3" t="inlineStr">
+        <is>
+          <t>765751002</t>
+        </is>
+      </c>
       <c r="K83" s="2" t="inlineStr"/>
     </row>
     <row r="84">
@@ -6218,7 +6214,7 @@
       <c r="I117" s="2" t="inlineStr"/>
       <c r="J117" s="3" t="inlineStr">
         <is>
-          <t>239796000, 410795001</t>
+          <t>410795001</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6320,7 +6316,7 @@
       <c r="I119" s="2" t="inlineStr"/>
       <c r="J119" s="3" t="inlineStr">
         <is>
-          <t>895454001, 25674000</t>
+          <t>895454001</t>
         </is>
       </c>
       <c r="K119" s="5" t="inlineStr">
@@ -6985,14 +6981,10 @@
       <c r="I132" s="2" t="inlineStr"/>
       <c r="J132" s="3" t="inlineStr">
         <is>
-          <t>201049004, 201048007</t>
-        </is>
-      </c>
-      <c r="K132" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>201048007</t>
+        </is>
+      </c>
+      <c r="K132" s="2" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -7250,7 +7242,7 @@
       <c r="I137" s="2" t="inlineStr"/>
       <c r="J137" s="3" t="inlineStr">
         <is>
-          <t>718213001, 1237194006</t>
+          <t>1237194006</t>
         </is>
       </c>
       <c r="K137" s="5" t="inlineStr">
@@ -7303,7 +7295,7 @@
       <c r="I138" s="2" t="inlineStr"/>
       <c r="J138" s="3" t="inlineStr">
         <is>
-          <t>871640001, 37217002</t>
+          <t>871640001</t>
         </is>
       </c>
       <c r="K138" s="5" t="inlineStr">
@@ -8943,7 +8935,7 @@
       <c r="I170" s="2" t="inlineStr"/>
       <c r="J170" s="3" t="inlineStr">
         <is>
-          <t>37042000, 9014002</t>
+          <t>9014002</t>
         </is>
       </c>
       <c r="K170" s="5" t="inlineStr">
@@ -9208,7 +9200,7 @@
       <c r="I175" s="2" t="inlineStr"/>
       <c r="J175" s="3" t="inlineStr">
         <is>
-          <t>356198000, 266261006</t>
+          <t>356198000</t>
         </is>
       </c>
       <c r="K175" s="5" t="inlineStr">
@@ -9261,7 +9253,7 @@
       <c r="I176" s="2" t="inlineStr"/>
       <c r="J176" s="3" t="inlineStr">
         <is>
-          <t>201736002, 67224007</t>
+          <t>201736002</t>
         </is>
       </c>
       <c r="K176" s="5" t="inlineStr">
@@ -9526,7 +9518,7 @@
       <c r="I181" s="2" t="inlineStr"/>
       <c r="J181" s="3" t="inlineStr">
         <is>
-          <t>194709000, 58718002</t>
+          <t>58718002</t>
         </is>
       </c>
       <c r="K181" s="5" t="inlineStr">
@@ -9738,7 +9730,7 @@
       <c r="I185" s="2" t="inlineStr"/>
       <c r="J185" s="3" t="inlineStr">
         <is>
-          <t>31541009, 238676008, 72470008</t>
+          <t>31541009</t>
         </is>
       </c>
       <c r="K185" s="5" t="inlineStr">

</xml_diff>